<commit_message>
Add standalone expanded feature statistics workbook
</commit_message>
<xml_diff>
--- a/语言特征说明.xlsx
+++ b/语言特征说明.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="语言特征说明" sheetId="1" r:id="R109db591c9f14d25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="语言特征说明" sheetId="1" r:id="R69e143b19f0e43ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,7 +37,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -67,6 +67,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF8064A2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6F5A8A"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -139,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -194,10 +199,10 @@
     <x:xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -210,6 +215,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -658,8 +666,8 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
-      <x:c r="A14" s="21" t="str">
-        <x:v>词汇丰富度</x:v>
+      <x:c r="A14" s="22" t="str">
+        <x:v>词汇集中度</x:v>
       </x:c>
       <x:c r="B14" s="18" t="n">
         <x:v>10</x:v>
@@ -668,7 +676,7 @@
         <x:v>篇内高频词前10位</x:v>
       </x:c>
       <x:c r="D14" s="17" t="str">
-        <x:v>篇内出现频率最高的10个非标点词形的token次数之和。报告形式：原始次数、每千汉字频率、比例。</x:v>
+        <x:v>篇内最高频10个非标点词形的覆盖程度；依据胡显耀TOP10概念改造为篇级词汇集中度指标，非原论文的子语料库统计。报告形式：原始次数、每千汉字频率、比例。</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
         <x:v>篇内频次最高的10个词</x:v>
@@ -758,7 +766,7 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
-      <x:c r="A19" s="22" t="str">
+      <x:c r="A19" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B19" s="18" t="n">
@@ -778,7 +786,7 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
-      <x:c r="A20" s="22" t="str">
+      <x:c r="A20" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B20" s="18" t="n">
@@ -798,7 +806,7 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
-      <x:c r="A21" s="22" t="str">
+      <x:c r="A21" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
@@ -818,7 +826,7 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
-      <x:c r="A22" s="22" t="str">
+      <x:c r="A22" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
@@ -838,7 +846,7 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
-      <x:c r="A23" s="22" t="str">
+      <x:c r="A23" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B23" s="18" t="n">
@@ -858,7 +866,7 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
-      <x:c r="A24" s="22" t="str">
+      <x:c r="A24" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B24" s="18" t="n">
@@ -878,7 +886,7 @@
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
-      <x:c r="A25" s="22" t="str">
+      <x:c r="A25" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
@@ -898,7 +906,7 @@
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
-      <x:c r="A26" s="22" t="str">
+      <x:c r="A26" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
@@ -918,7 +926,7 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
-      <x:c r="A27" s="22" t="str">
+      <x:c r="A27" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
@@ -938,7 +946,7 @@
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
-      <x:c r="A28" s="22" t="str">
+      <x:c r="A28" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
@@ -958,7 +966,7 @@
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
-      <x:c r="A29" s="22" t="str">
+      <x:c r="A29" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B29" s="18" t="n">
@@ -978,7 +986,7 @@
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
-      <x:c r="A30" s="22" t="str">
+      <x:c r="A30" s="23" t="str">
         <x:v>词汇密度与词长</x:v>
       </x:c>
       <x:c r="B30" s="18" t="n">
@@ -998,7 +1006,7 @@
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
-      <x:c r="A31" s="23" t="str">
+      <x:c r="A31" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
@@ -1018,7 +1026,7 @@
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
-      <x:c r="A32" s="23" t="str">
+      <x:c r="A32" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
@@ -1038,7 +1046,7 @@
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
-      <x:c r="A33" s="23" t="str">
+      <x:c r="A33" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
@@ -1058,7 +1066,7 @@
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
-      <x:c r="A34" s="23" t="str">
+      <x:c r="A34" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B34" s="18" t="n">
@@ -1078,7 +1086,7 @@
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
-      <x:c r="A35" s="23" t="str">
+      <x:c r="A35" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B35" s="18" t="n">
@@ -1098,7 +1106,7 @@
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
-      <x:c r="A36" s="23" t="str">
+      <x:c r="A36" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
@@ -1118,7 +1126,7 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
-      <x:c r="A37" s="23" t="str">
+      <x:c r="A37" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
@@ -1138,7 +1146,7 @@
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
-      <x:c r="A38" s="23" t="str">
+      <x:c r="A38" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
@@ -1158,7 +1166,7 @@
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
-      <x:c r="A39" s="23" t="str">
+      <x:c r="A39" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
@@ -1178,7 +1186,7 @@
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
-      <x:c r="A40" s="23" t="str">
+      <x:c r="A40" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B40" s="18" t="n">
@@ -1198,7 +1206,7 @@
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
-      <x:c r="A41" s="23" t="str">
+      <x:c r="A41" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B41" s="18" t="n">
@@ -1218,7 +1226,7 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
-      <x:c r="A42" s="23" t="str">
+      <x:c r="A42" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
@@ -1238,7 +1246,7 @@
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
-      <x:c r="A43" s="23" t="str">
+      <x:c r="A43" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B43" s="18" t="n">
@@ -1258,7 +1266,7 @@
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
-      <x:c r="A44" s="23" t="str">
+      <x:c r="A44" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B44" s="18" t="n">
@@ -1278,7 +1286,7 @@
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
-      <x:c r="A45" s="23" t="str">
+      <x:c r="A45" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B45" s="18" t="n">
@@ -1298,7 +1306,7 @@
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
-      <x:c r="A46" s="23" t="str">
+      <x:c r="A46" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B46" s="18" t="n">
@@ -1318,7 +1326,7 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
-      <x:c r="A47" s="23" t="str">
+      <x:c r="A47" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B47" s="18" t="n">
@@ -1338,7 +1346,7 @@
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
-      <x:c r="A48" s="23" t="str">
+      <x:c r="A48" s="24" t="str">
         <x:v>句段结构</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
@@ -1358,7 +1366,7 @@
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
-      <x:c r="A49" s="24" t="str">
+      <x:c r="A49" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
@@ -1378,7 +1386,7 @@
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
-      <x:c r="A50" s="24" t="str">
+      <x:c r="A50" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
@@ -1398,7 +1406,7 @@
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
-      <x:c r="A51" s="24" t="str">
+      <x:c r="A51" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
@@ -1418,7 +1426,7 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
-      <x:c r="A52" s="24" t="str">
+      <x:c r="A52" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B52" s="18" t="n">
@@ -1438,7 +1446,7 @@
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
-      <x:c r="A53" s="24" t="str">
+      <x:c r="A53" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B53" s="18" t="n">
@@ -1458,7 +1466,7 @@
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
-      <x:c r="A54" s="24" t="str">
+      <x:c r="A54" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B54" s="18" t="n">
@@ -1478,7 +1486,7 @@
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
-      <x:c r="A55" s="24" t="str">
+      <x:c r="A55" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B55" s="18" t="n">
@@ -1498,7 +1506,7 @@
       </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
-      <x:c r="A56" s="24" t="str">
+      <x:c r="A56" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B56" s="18" t="n">
@@ -1518,7 +1526,7 @@
       </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
-      <x:c r="A57" s="24" t="str">
+      <x:c r="A57" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B57" s="18" t="n">
@@ -1538,7 +1546,7 @@
       </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
-      <x:c r="A58" s="24" t="str">
+      <x:c r="A58" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B58" s="18" t="n">
@@ -1558,7 +1566,7 @@
       </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
-      <x:c r="A59" s="24" t="str">
+      <x:c r="A59" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B59" s="18" t="n">
@@ -1578,7 +1586,7 @@
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
-      <x:c r="A60" s="24" t="str">
+      <x:c r="A60" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B60" s="18" t="n">
@@ -1598,7 +1606,7 @@
       </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
-      <x:c r="A61" s="24" t="str">
+      <x:c r="A61" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B61" s="18" t="n">
@@ -1618,7 +1626,7 @@
       </x:c>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
-      <x:c r="A62" s="24" t="str">
+      <x:c r="A62" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B62" s="18" t="n">
@@ -1638,7 +1646,7 @@
       </x:c>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
-      <x:c r="A63" s="24" t="str">
+      <x:c r="A63" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B63" s="18" t="n">
@@ -1658,7 +1666,7 @@
       </x:c>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
-      <x:c r="A64" s="24" t="str">
+      <x:c r="A64" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B64" s="18" t="n">
@@ -1678,7 +1686,7 @@
       </x:c>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
-      <x:c r="A65" s="24" t="str">
+      <x:c r="A65" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B65" s="18" t="n">
@@ -1698,7 +1706,7 @@
       </x:c>
     </x:row>
     <x:row r="66" ht="42" customHeight="1">
-      <x:c r="A66" s="24" t="str">
+      <x:c r="A66" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B66" s="18" t="n">
@@ -1718,7 +1726,7 @@
       </x:c>
     </x:row>
     <x:row r="67" ht="42" customHeight="1">
-      <x:c r="A67" s="24" t="str">
+      <x:c r="A67" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B67" s="18" t="n">
@@ -1738,7 +1746,7 @@
       </x:c>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
-      <x:c r="A68" s="24" t="str">
+      <x:c r="A68" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B68" s="18" t="n">
@@ -1758,7 +1766,7 @@
       </x:c>
     </x:row>
     <x:row r="69" ht="42" customHeight="1">
-      <x:c r="A69" s="24" t="str">
+      <x:c r="A69" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B69" s="18" t="n">
@@ -1778,7 +1786,7 @@
       </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
-      <x:c r="A70" s="24" t="str">
+      <x:c r="A70" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B70" s="18" t="n">
@@ -1798,7 +1806,7 @@
       </x:c>
     </x:row>
     <x:row r="71" ht="42" customHeight="1">
-      <x:c r="A71" s="24" t="str">
+      <x:c r="A71" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B71" s="18" t="n">
@@ -1818,7 +1826,7 @@
       </x:c>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
-      <x:c r="A72" s="24" t="str">
+      <x:c r="A72" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B72" s="18" t="n">
@@ -1838,7 +1846,7 @@
       </x:c>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
-      <x:c r="A73" s="24" t="str">
+      <x:c r="A73" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B73" s="18" t="n">
@@ -1858,7 +1866,7 @@
       </x:c>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
-      <x:c r="A74" s="24" t="str">
+      <x:c r="A74" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B74" s="18" t="n">
@@ -1878,7 +1886,7 @@
       </x:c>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
-      <x:c r="A75" s="24" t="str">
+      <x:c r="A75" s="25" t="str">
         <x:v>词性</x:v>
       </x:c>
       <x:c r="B75" s="18" t="n">
@@ -1898,7 +1906,7 @@
       </x:c>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
-      <x:c r="A76" s="25" t="str">
+      <x:c r="A76" s="26" t="str">
         <x:v>熟语</x:v>
       </x:c>
       <x:c r="B76" s="18" t="n">
@@ -1918,7 +1926,7 @@
       </x:c>
     </x:row>
     <x:row r="77" ht="42" customHeight="1">
-      <x:c r="A77" s="25" t="str">
+      <x:c r="A77" s="26" t="str">
         <x:v>熟语</x:v>
       </x:c>
       <x:c r="B77" s="18" t="n">
@@ -1938,7 +1946,7 @@
       </x:c>
     </x:row>
     <x:row r="78" ht="42" customHeight="1">
-      <x:c r="A78" s="25" t="str">
+      <x:c r="A78" s="26" t="str">
         <x:v>熟语</x:v>
       </x:c>
       <x:c r="B78" s="18" t="n">
@@ -1958,7 +1966,7 @@
       </x:c>
     </x:row>
     <x:row r="79" ht="42" customHeight="1">
-      <x:c r="A79" s="25" t="str">
+      <x:c r="A79" s="26" t="str">
         <x:v>熟语</x:v>
       </x:c>
       <x:c r="B79" s="18" t="n">
@@ -1978,7 +1986,7 @@
       </x:c>
     </x:row>
     <x:row r="80" ht="42" customHeight="1">
-      <x:c r="A80" s="25" t="str">
+      <x:c r="A80" s="26" t="str">
         <x:v>熟语</x:v>
       </x:c>
       <x:c r="B80" s="18" t="n">
@@ -1998,7 +2006,7 @@
       </x:c>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
-      <x:c r="A81" s="25" t="str">
+      <x:c r="A81" s="26" t="str">
         <x:v>熟语</x:v>
       </x:c>
       <x:c r="B81" s="18" t="n">
@@ -2018,7 +2026,7 @@
       </x:c>
     </x:row>
     <x:row r="82" ht="42" customHeight="1">
-      <x:c r="A82" s="26" t="str">
+      <x:c r="A82" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B82" s="18" t="n">
@@ -2038,7 +2046,7 @@
       </x:c>
     </x:row>
     <x:row r="83" ht="42" customHeight="1">
-      <x:c r="A83" s="26" t="str">
+      <x:c r="A83" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B83" s="18" t="n">
@@ -2058,7 +2066,7 @@
       </x:c>
     </x:row>
     <x:row r="84" ht="42" customHeight="1">
-      <x:c r="A84" s="26" t="str">
+      <x:c r="A84" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B84" s="18" t="n">
@@ -2078,7 +2086,7 @@
       </x:c>
     </x:row>
     <x:row r="85" ht="42" customHeight="1">
-      <x:c r="A85" s="26" t="str">
+      <x:c r="A85" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B85" s="18" t="n">
@@ -2098,7 +2106,7 @@
       </x:c>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
-      <x:c r="A86" s="26" t="str">
+      <x:c r="A86" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B86" s="18" t="n">
@@ -2118,7 +2126,7 @@
       </x:c>
     </x:row>
     <x:row r="87" ht="42" customHeight="1">
-      <x:c r="A87" s="26" t="str">
+      <x:c r="A87" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B87" s="18" t="n">
@@ -2138,7 +2146,7 @@
       </x:c>
     </x:row>
     <x:row r="88" ht="42" customHeight="1">
-      <x:c r="A88" s="26" t="str">
+      <x:c r="A88" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B88" s="18" t="n">
@@ -2158,7 +2166,7 @@
       </x:c>
     </x:row>
     <x:row r="89" ht="42" customHeight="1">
-      <x:c r="A89" s="26" t="str">
+      <x:c r="A89" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B89" s="18" t="n">
@@ -2178,7 +2186,7 @@
       </x:c>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
-      <x:c r="A90" s="26" t="str">
+      <x:c r="A90" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B90" s="18" t="n">
@@ -2198,7 +2206,7 @@
       </x:c>
     </x:row>
     <x:row r="91" ht="42" customHeight="1">
-      <x:c r="A91" s="26" t="str">
+      <x:c r="A91" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B91" s="18" t="n">
@@ -2218,7 +2226,7 @@
       </x:c>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
-      <x:c r="A92" s="26" t="str">
+      <x:c r="A92" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B92" s="18" t="n">
@@ -2238,7 +2246,7 @@
       </x:c>
     </x:row>
     <x:row r="93" ht="42" customHeight="1">
-      <x:c r="A93" s="26" t="str">
+      <x:c r="A93" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B93" s="18" t="n">
@@ -2258,7 +2266,7 @@
       </x:c>
     </x:row>
     <x:row r="94" ht="42" customHeight="1">
-      <x:c r="A94" s="26" t="str">
+      <x:c r="A94" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B94" s="18" t="n">
@@ -2278,7 +2286,7 @@
       </x:c>
     </x:row>
     <x:row r="95" ht="42" customHeight="1">
-      <x:c r="A95" s="26" t="str">
+      <x:c r="A95" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B95" s="18" t="n">
@@ -2298,7 +2306,7 @@
       </x:c>
     </x:row>
     <x:row r="96" ht="42" customHeight="1">
-      <x:c r="A96" s="26" t="str">
+      <x:c r="A96" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B96" s="18" t="n">
@@ -2318,7 +2326,7 @@
       </x:c>
     </x:row>
     <x:row r="97" ht="42" customHeight="1">
-      <x:c r="A97" s="26" t="str">
+      <x:c r="A97" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B97" s="18" t="n">
@@ -2338,7 +2346,7 @@
       </x:c>
     </x:row>
     <x:row r="98" ht="42" customHeight="1">
-      <x:c r="A98" s="26" t="str">
+      <x:c r="A98" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B98" s="18" t="n">
@@ -2358,7 +2366,7 @@
       </x:c>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
-      <x:c r="A99" s="26" t="str">
+      <x:c r="A99" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B99" s="18" t="n">
@@ -2378,7 +2386,7 @@
       </x:c>
     </x:row>
     <x:row r="100" ht="42" customHeight="1">
-      <x:c r="A100" s="26" t="str">
+      <x:c r="A100" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B100" s="18" t="n">
@@ -2398,7 +2406,7 @@
       </x:c>
     </x:row>
     <x:row r="101" ht="42" customHeight="1">
-      <x:c r="A101" s="26" t="str">
+      <x:c r="A101" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B101" s="18" t="n">
@@ -2418,7 +2426,7 @@
       </x:c>
     </x:row>
     <x:row r="102" ht="42" customHeight="1">
-      <x:c r="A102" s="26" t="str">
+      <x:c r="A102" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B102" s="18" t="n">
@@ -2438,7 +2446,7 @@
       </x:c>
     </x:row>
     <x:row r="103" ht="42" customHeight="1">
-      <x:c r="A103" s="26" t="str">
+      <x:c r="A103" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B103" s="18" t="n">
@@ -2458,7 +2466,7 @@
       </x:c>
     </x:row>
     <x:row r="104" ht="42" customHeight="1">
-      <x:c r="A104" s="26" t="str">
+      <x:c r="A104" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B104" s="18" t="n">
@@ -2478,7 +2486,7 @@
       </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
-      <x:c r="A105" s="26" t="str">
+      <x:c r="A105" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B105" s="18" t="n">
@@ -2498,7 +2506,7 @@
       </x:c>
     </x:row>
     <x:row r="106" ht="42" customHeight="1">
-      <x:c r="A106" s="26" t="str">
+      <x:c r="A106" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B106" s="18" t="n">
@@ -2518,7 +2526,7 @@
       </x:c>
     </x:row>
     <x:row r="107" ht="42" customHeight="1">
-      <x:c r="A107" s="26" t="str">
+      <x:c r="A107" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B107" s="18" t="n">
@@ -2538,7 +2546,7 @@
       </x:c>
     </x:row>
     <x:row r="108" ht="42" customHeight="1">
-      <x:c r="A108" s="26" t="str">
+      <x:c r="A108" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B108" s="18" t="n">
@@ -2558,7 +2566,7 @@
       </x:c>
     </x:row>
     <x:row r="109" ht="42" customHeight="1">
-      <x:c r="A109" s="26" t="str">
+      <x:c r="A109" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B109" s="18" t="n">
@@ -2578,7 +2586,7 @@
       </x:c>
     </x:row>
     <x:row r="110" ht="42" customHeight="1">
-      <x:c r="A110" s="26" t="str">
+      <x:c r="A110" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B110" s="18" t="n">
@@ -2598,7 +2606,7 @@
       </x:c>
     </x:row>
     <x:row r="111" ht="42" customHeight="1">
-      <x:c r="A111" s="26" t="str">
+      <x:c r="A111" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B111" s="18" t="n">
@@ -2618,7 +2626,7 @@
       </x:c>
     </x:row>
     <x:row r="112" ht="42" customHeight="1">
-      <x:c r="A112" s="26" t="str">
+      <x:c r="A112" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B112" s="18" t="n">
@@ -2638,7 +2646,7 @@
       </x:c>
     </x:row>
     <x:row r="113" ht="42" customHeight="1">
-      <x:c r="A113" s="26" t="str">
+      <x:c r="A113" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B113" s="18" t="n">
@@ -2658,7 +2666,7 @@
       </x:c>
     </x:row>
     <x:row r="114" ht="42" customHeight="1">
-      <x:c r="A114" s="26" t="str">
+      <x:c r="A114" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B114" s="18" t="n">
@@ -2678,7 +2686,7 @@
       </x:c>
     </x:row>
     <x:row r="115" ht="42" customHeight="1">
-      <x:c r="A115" s="26" t="str">
+      <x:c r="A115" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B115" s="18" t="n">
@@ -2698,7 +2706,7 @@
       </x:c>
     </x:row>
     <x:row r="116" ht="42" customHeight="1">
-      <x:c r="A116" s="26" t="str">
+      <x:c r="A116" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B116" s="18" t="n">
@@ -2718,7 +2726,7 @@
       </x:c>
     </x:row>
     <x:row r="117" ht="42" customHeight="1">
-      <x:c r="A117" s="26" t="str">
+      <x:c r="A117" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B117" s="18" t="n">
@@ -2738,7 +2746,7 @@
       </x:c>
     </x:row>
     <x:row r="118" ht="42" customHeight="1">
-      <x:c r="A118" s="26" t="str">
+      <x:c r="A118" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B118" s="18" t="n">
@@ -2758,7 +2766,7 @@
       </x:c>
     </x:row>
     <x:row r="119" ht="42" customHeight="1">
-      <x:c r="A119" s="26" t="str">
+      <x:c r="A119" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B119" s="18" t="n">
@@ -2778,7 +2786,7 @@
       </x:c>
     </x:row>
     <x:row r="120" ht="42" customHeight="1">
-      <x:c r="A120" s="26" t="str">
+      <x:c r="A120" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B120" s="18" t="n">
@@ -2798,7 +2806,7 @@
       </x:c>
     </x:row>
     <x:row r="121" ht="42" customHeight="1">
-      <x:c r="A121" s="26" t="str">
+      <x:c r="A121" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B121" s="18" t="n">
@@ -2818,7 +2826,7 @@
       </x:c>
     </x:row>
     <x:row r="122" ht="42" customHeight="1">
-      <x:c r="A122" s="26" t="str">
+      <x:c r="A122" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B122" s="18" t="n">
@@ -2838,7 +2846,7 @@
       </x:c>
     </x:row>
     <x:row r="123" ht="42" customHeight="1">
-      <x:c r="A123" s="26" t="str">
+      <x:c r="A123" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B123" s="18" t="n">
@@ -2858,7 +2866,7 @@
       </x:c>
     </x:row>
     <x:row r="124" ht="42" customHeight="1">
-      <x:c r="A124" s="26" t="str">
+      <x:c r="A124" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B124" s="18" t="n">
@@ -2878,7 +2886,7 @@
       </x:c>
     </x:row>
     <x:row r="125" ht="42" customHeight="1">
-      <x:c r="A125" s="26" t="str">
+      <x:c r="A125" s="27" t="str">
         <x:v>语法标记</x:v>
       </x:c>
       <x:c r="B125" s="18" t="n">
@@ -2898,7 +2906,7 @@
       </x:c>
     </x:row>
     <x:row r="126" ht="42" customHeight="1">
-      <x:c r="A126" s="27" t="str">
+      <x:c r="A126" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B126" s="18" t="n">
@@ -2918,7 +2926,7 @@
       </x:c>
     </x:row>
     <x:row r="127" ht="42" customHeight="1">
-      <x:c r="A127" s="27" t="str">
+      <x:c r="A127" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B127" s="18" t="n">
@@ -2938,7 +2946,7 @@
       </x:c>
     </x:row>
     <x:row r="128" ht="42" customHeight="1">
-      <x:c r="A128" s="27" t="str">
+      <x:c r="A128" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B128" s="18" t="n">
@@ -2958,7 +2966,7 @@
       </x:c>
     </x:row>
     <x:row r="129" ht="42" customHeight="1">
-      <x:c r="A129" s="27" t="str">
+      <x:c r="A129" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B129" s="18" t="n">
@@ -2978,7 +2986,7 @@
       </x:c>
     </x:row>
     <x:row r="130" ht="42" customHeight="1">
-      <x:c r="A130" s="27" t="str">
+      <x:c r="A130" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B130" s="18" t="n">
@@ -2998,7 +3006,7 @@
       </x:c>
     </x:row>
     <x:row r="131" ht="42" customHeight="1">
-      <x:c r="A131" s="27" t="str">
+      <x:c r="A131" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B131" s="18" t="n">
@@ -3018,7 +3026,7 @@
       </x:c>
     </x:row>
     <x:row r="132" ht="42" customHeight="1">
-      <x:c r="A132" s="27" t="str">
+      <x:c r="A132" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B132" s="18" t="n">
@@ -3038,7 +3046,7 @@
       </x:c>
     </x:row>
     <x:row r="133" ht="42" customHeight="1">
-      <x:c r="A133" s="27" t="str">
+      <x:c r="A133" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B133" s="18" t="n">
@@ -3058,7 +3066,7 @@
       </x:c>
     </x:row>
     <x:row r="134" ht="42" customHeight="1">
-      <x:c r="A134" s="27" t="str">
+      <x:c r="A134" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B134" s="18" t="n">
@@ -3078,7 +3086,7 @@
       </x:c>
     </x:row>
     <x:row r="135" ht="42" customHeight="1">
-      <x:c r="A135" s="27" t="str">
+      <x:c r="A135" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B135" s="18" t="n">
@@ -3098,7 +3106,7 @@
       </x:c>
     </x:row>
     <x:row r="136" ht="42" customHeight="1">
-      <x:c r="A136" s="27" t="str">
+      <x:c r="A136" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B136" s="18" t="n">
@@ -3118,7 +3126,7 @@
       </x:c>
     </x:row>
     <x:row r="137" ht="42" customHeight="1">
-      <x:c r="A137" s="27" t="str">
+      <x:c r="A137" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B137" s="18" t="n">
@@ -3138,7 +3146,7 @@
       </x:c>
     </x:row>
     <x:row r="138" ht="42" customHeight="1">
-      <x:c r="A138" s="27" t="str">
+      <x:c r="A138" s="28" t="str">
         <x:v>复句关系</x:v>
       </x:c>
       <x:c r="B138" s="18" t="n">
@@ -3158,7 +3166,7 @@
       </x:c>
     </x:row>
     <x:row r="139" ht="42" customHeight="1">
-      <x:c r="A139" s="28" t="str">
+      <x:c r="A139" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B139" s="18" t="n">
@@ -3178,7 +3186,7 @@
       </x:c>
     </x:row>
     <x:row r="140" ht="42" customHeight="1">
-      <x:c r="A140" s="28" t="str">
+      <x:c r="A140" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B140" s="18" t="n">
@@ -3198,7 +3206,7 @@
       </x:c>
     </x:row>
     <x:row r="141" ht="42" customHeight="1">
-      <x:c r="A141" s="28" t="str">
+      <x:c r="A141" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B141" s="18" t="n">
@@ -3218,7 +3226,7 @@
       </x:c>
     </x:row>
     <x:row r="142" ht="42" customHeight="1">
-      <x:c r="A142" s="28" t="str">
+      <x:c r="A142" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B142" s="18" t="n">
@@ -3238,7 +3246,7 @@
       </x:c>
     </x:row>
     <x:row r="143" ht="42" customHeight="1">
-      <x:c r="A143" s="28" t="str">
+      <x:c r="A143" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B143" s="18" t="n">
@@ -3258,7 +3266,7 @@
       </x:c>
     </x:row>
     <x:row r="144" ht="42" customHeight="1">
-      <x:c r="A144" s="28" t="str">
+      <x:c r="A144" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B144" s="18" t="n">
@@ -3278,7 +3286,7 @@
       </x:c>
     </x:row>
     <x:row r="145" ht="42" customHeight="1">
-      <x:c r="A145" s="28" t="str">
+      <x:c r="A145" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B145" s="18" t="n">
@@ -3298,7 +3306,7 @@
       </x:c>
     </x:row>
     <x:row r="146" ht="42" customHeight="1">
-      <x:c r="A146" s="28" t="str">
+      <x:c r="A146" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B146" s="18" t="n">
@@ -3318,7 +3326,7 @@
       </x:c>
     </x:row>
     <x:row r="147" ht="42" customHeight="1">
-      <x:c r="A147" s="28" t="str">
+      <x:c r="A147" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B147" s="18" t="n">
@@ -3338,7 +3346,7 @@
       </x:c>
     </x:row>
     <x:row r="148" ht="42" customHeight="1">
-      <x:c r="A148" s="28" t="str">
+      <x:c r="A148" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B148" s="18" t="n">
@@ -3358,7 +3366,7 @@
       </x:c>
     </x:row>
     <x:row r="149" ht="42" customHeight="1">
-      <x:c r="A149" s="28" t="str">
+      <x:c r="A149" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B149" s="18" t="n">
@@ -3378,7 +3386,7 @@
       </x:c>
     </x:row>
     <x:row r="150" ht="42" customHeight="1">
-      <x:c r="A150" s="28" t="str">
+      <x:c r="A150" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B150" s="18" t="n">
@@ -3398,7 +3406,7 @@
       </x:c>
     </x:row>
     <x:row r="151" ht="42" customHeight="1">
-      <x:c r="A151" s="28" t="str">
+      <x:c r="A151" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B151" s="18" t="n">
@@ -3418,7 +3426,7 @@
       </x:c>
     </x:row>
     <x:row r="152" ht="42" customHeight="1">
-      <x:c r="A152" s="28" t="str">
+      <x:c r="A152" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B152" s="18" t="n">
@@ -3438,7 +3446,7 @@
       </x:c>
     </x:row>
     <x:row r="153" ht="42" customHeight="1">
-      <x:c r="A153" s="28" t="str">
+      <x:c r="A153" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B153" s="18" t="n">
@@ -3458,7 +3466,7 @@
       </x:c>
     </x:row>
     <x:row r="154" ht="42" customHeight="1">
-      <x:c r="A154" s="28" t="str">
+      <x:c r="A154" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B154" s="18" t="n">
@@ -3478,7 +3486,7 @@
       </x:c>
     </x:row>
     <x:row r="155" ht="42" customHeight="1">
-      <x:c r="A155" s="28" t="str">
+      <x:c r="A155" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B155" s="18" t="n">
@@ -3498,7 +3506,7 @@
       </x:c>
     </x:row>
     <x:row r="156" ht="42" customHeight="1">
-      <x:c r="A156" s="28" t="str">
+      <x:c r="A156" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B156" s="18" t="n">
@@ -3518,7 +3526,7 @@
       </x:c>
     </x:row>
     <x:row r="157" ht="42" customHeight="1">
-      <x:c r="A157" s="28" t="str">
+      <x:c r="A157" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B157" s="18" t="n">
@@ -3538,7 +3546,7 @@
       </x:c>
     </x:row>
     <x:row r="158" ht="42" customHeight="1">
-      <x:c r="A158" s="28" t="str">
+      <x:c r="A158" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B158" s="18" t="n">
@@ -3558,7 +3566,7 @@
       </x:c>
     </x:row>
     <x:row r="159" ht="42" customHeight="1">
-      <x:c r="A159" s="28" t="str">
+      <x:c r="A159" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B159" s="18" t="n">
@@ -3578,7 +3586,7 @@
       </x:c>
     </x:row>
     <x:row r="160" ht="42" customHeight="1">
-      <x:c r="A160" s="28" t="str">
+      <x:c r="A160" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B160" s="18" t="n">
@@ -3598,7 +3606,7 @@
       </x:c>
     </x:row>
     <x:row r="161" ht="42" customHeight="1">
-      <x:c r="A161" s="28" t="str">
+      <x:c r="A161" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B161" s="18" t="n">
@@ -3618,7 +3626,7 @@
       </x:c>
     </x:row>
     <x:row r="162" ht="42" customHeight="1">
-      <x:c r="A162" s="28" t="str">
+      <x:c r="A162" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B162" s="18" t="n">
@@ -3638,7 +3646,7 @@
       </x:c>
     </x:row>
     <x:row r="163" ht="42" customHeight="1">
-      <x:c r="A163" s="28" t="str">
+      <x:c r="A163" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B163" s="18" t="n">
@@ -3658,7 +3666,7 @@
       </x:c>
     </x:row>
     <x:row r="164" ht="42" customHeight="1">
-      <x:c r="A164" s="28" t="str">
+      <x:c r="A164" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B164" s="18" t="n">
@@ -3678,7 +3686,7 @@
       </x:c>
     </x:row>
     <x:row r="165" ht="42" customHeight="1">
-      <x:c r="A165" s="28" t="str">
+      <x:c r="A165" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B165" s="18" t="n">
@@ -3698,7 +3706,7 @@
       </x:c>
     </x:row>
     <x:row r="166" ht="42" customHeight="1">
-      <x:c r="A166" s="28" t="str">
+      <x:c r="A166" s="29" t="str">
         <x:v>记叙描写</x:v>
       </x:c>
       <x:c r="B166" s="18" t="n">
@@ -3718,7 +3726,7 @@
       </x:c>
     </x:row>
     <x:row r="167" ht="42" customHeight="1">
-      <x:c r="A167" s="29" t="str">
+      <x:c r="A167" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B167" s="18" t="n">
@@ -3738,7 +3746,7 @@
       </x:c>
     </x:row>
     <x:row r="168" ht="42" customHeight="1">
-      <x:c r="A168" s="29" t="str">
+      <x:c r="A168" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B168" s="18" t="n">
@@ -3758,7 +3766,7 @@
       </x:c>
     </x:row>
     <x:row r="169" ht="42" customHeight="1">
-      <x:c r="A169" s="29" t="str">
+      <x:c r="A169" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B169" s="18" t="n">
@@ -3778,7 +3786,7 @@
       </x:c>
     </x:row>
     <x:row r="170" ht="42" customHeight="1">
-      <x:c r="A170" s="29" t="str">
+      <x:c r="A170" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B170" s="18" t="n">
@@ -3798,7 +3806,7 @@
       </x:c>
     </x:row>
     <x:row r="171" ht="42" customHeight="1">
-      <x:c r="A171" s="29" t="str">
+      <x:c r="A171" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B171" s="18" t="n">
@@ -3818,7 +3826,7 @@
       </x:c>
     </x:row>
     <x:row r="172" ht="42" customHeight="1">
-      <x:c r="A172" s="29" t="str">
+      <x:c r="A172" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B172" s="18" t="n">
@@ -3838,7 +3846,7 @@
       </x:c>
     </x:row>
     <x:row r="173" ht="42" customHeight="1">
-      <x:c r="A173" s="29" t="str">
+      <x:c r="A173" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B173" s="18" t="n">
@@ -3858,7 +3866,7 @@
       </x:c>
     </x:row>
     <x:row r="174" ht="42" customHeight="1">
-      <x:c r="A174" s="29" t="str">
+      <x:c r="A174" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B174" s="18" t="n">
@@ -3878,7 +3886,7 @@
       </x:c>
     </x:row>
     <x:row r="175" ht="42" customHeight="1">
-      <x:c r="A175" s="29" t="str">
+      <x:c r="A175" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B175" s="18" t="n">
@@ -3898,7 +3906,7 @@
       </x:c>
     </x:row>
     <x:row r="176" ht="42" customHeight="1">
-      <x:c r="A176" s="29" t="str">
+      <x:c r="A176" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B176" s="18" t="n">
@@ -3918,7 +3926,7 @@
       </x:c>
     </x:row>
     <x:row r="177" ht="42" customHeight="1">
-      <x:c r="A177" s="29" t="str">
+      <x:c r="A177" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B177" s="18" t="n">
@@ -3938,7 +3946,7 @@
       </x:c>
     </x:row>
     <x:row r="178" ht="42" customHeight="1">
-      <x:c r="A178" s="29" t="str">
+      <x:c r="A178" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B178" s="18" t="n">
@@ -3958,7 +3966,7 @@
       </x:c>
     </x:row>
     <x:row r="179" ht="42" customHeight="1">
-      <x:c r="A179" s="29" t="str">
+      <x:c r="A179" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B179" s="18" t="n">
@@ -3978,7 +3986,7 @@
       </x:c>
     </x:row>
     <x:row r="180" ht="42" customHeight="1">
-      <x:c r="A180" s="29" t="str">
+      <x:c r="A180" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B180" s="18" t="n">
@@ -3998,7 +4006,7 @@
       </x:c>
     </x:row>
     <x:row r="181" ht="42" customHeight="1">
-      <x:c r="A181" s="29" t="str">
+      <x:c r="A181" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B181" s="18" t="n">
@@ -4018,7 +4026,7 @@
       </x:c>
     </x:row>
     <x:row r="182" ht="42" customHeight="1">
-      <x:c r="A182" s="29" t="str">
+      <x:c r="A182" s="30" t="str">
         <x:v>HSK</x:v>
       </x:c>
       <x:c r="B182" s="18" t="n">
@@ -4044,7 +4052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bfc0dd327514971"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cdff8519f784e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>